<commit_message>
HT ride kit: missed-leg table, verify list, booking list, start day; attempt_prep for HT
docs/ht_itinerary.xlsx gains four sheets. If you miss a leg: replay from the boarding stop one minute
after the bus left (HT's remaining stops, with each leg's states pinned so a later bus cannot skip one)
and, separately, the same chain N days later checked trip by trip; keep the earlier finish. Five misses
cost 0, most 24 h, the Memphis morning ~20 h, the last leg 14.4 h. Verify: hand-entered legs and the
router's local-transit proxies. Book ahead: 30 reservable legs with dates for a Monday start. Start
day: Monday recommended (Mon-Wed 230.10 h; Thu puts Memphis on Saturday; Sat/Sun lose Missouri).
Leaf script; nothing imports it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ht_itinerary.xlsx
+++ b/docs/ht_itinerary.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="HT itinerary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Start day" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="If you miss a leg" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Verify" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Book ahead" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +54,16 @@
         <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -64,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +88,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3012,13 +3028,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3039,14 +3055,14 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Memphis on real MATA</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mon / Tue / Wed</t>
+          <t>Monday (recommended)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3056,19 +3072,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed / Thu / Fri</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>yes: Walker 04:30 reaches the bridge for the 05:45 walk</t>
+          <t>Memphis on weekday MATA (Walker 04:30 to the bridge); Chicago on a Wednesday, when the extra Four Winds shuttles run (from Oct 28)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Tuesday / Wednesday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3078,19 +3094,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Thursday / Friday</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>no: first useful MATA is 07:00; needs a taxi from the terminal</t>
+          <t>same chain, weekday Memphis</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3100,30 +3116,3072 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sun</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>not checked</t>
+          <t>no MATA early enough on Saturday: taxi from the Greyhound terminal to the bridge</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sat / Sun</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>chain breaks</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>230.10 h</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>a non-daily service in the chain</t>
+          <t>Sunday MATA not checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday / Sunday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>misses Missouri</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>the Sioux Falls dead-time ride does not reach Missouri on those days; a detour would be needed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>missed</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>next best finish</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>cost h</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>recovery starts with</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>d5 Mon 06:40 Dartmouth Coach</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>d5 Mon 10:00 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>d5 Mon 12:30 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>d5 Mon 15:10 Amtrak</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>d6 Tue 00:30 FlixBus-us</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>d6 Tue 01:20 Greyhound-us: Washington Union Station -&gt; Raleigh Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>d6 Tue 12:05 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>d6 Tue 17:05 Greyhound-us: Augusta -&gt; Lugoff (Shiv Mart)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>d6 Tue 15:15 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Charlotte Bus Station</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>d6 Tue 19:00 Greyhound-us: Lugoff (Shiv Mart) -&gt; Charlotte Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>d6 Tue 17:45 Barons Bus Lines</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>d7 Wed 02:50 Greyhound-us: Charlotte Bus Station -&gt; Columbus (E Mound St)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>d7 Wed 06:15 Barons Bus Lines</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Michigan City</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>d7 Wed 09:45 FlixBus-us: Columbus (E Rich St) -&gt; Chicago Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>d7 Wed 12:38 Michian City Transit</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Marquette Mall Transfer Point</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E 4th Street/Franklin Street                                       </t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>d14 Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>d7 Wed 12:56 Michian City Transit: Horizon Bank/MyEyeDr -&gt; Library</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>d7 Wed 13:51 Michian City Transit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E 4th Street/Franklin Street                                       </t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Als Karwick</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>d14 Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>d7 Wed 14:51 Michian City Transit: E 4th Street/Franklin Street                                        -&gt; Als Karwick</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>d7 Wed 17:39 Northern Indiana Commuter Transportation District</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Carroll Ave. (Michigan City)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Museum Campus/11th St.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>d8 Thu 04:08 Northern Indiana Commuter Transportation District: Carroll Ave. (Michigan City) -&gt; Museum Campus/11th St.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>d7 Wed 22:00 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>d14 Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>d8 Thu 00:30 Greyhound-us: Chicago Bus Station -&gt; Minneapolis Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>d8 Thu 10:35 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>d8 Thu 11:35 Jefferson Lines: Minneapolis -&gt; Brainerd</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>d8 Thu 15:50 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>d8 Thu 16:40 Jefferson Lines: Fargo -&gt; Minneapolis</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>d8 Thu 20:05 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>d9 Fri 20:05 Jefferson Lines: Sioux Falls -&gt; Maryville</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>d9 Fri 03:25 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>d10 Sat 03:25 Jefferson Lines: Maryville -&gt; Sioux Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>d9 Fri 12:40 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>d9 Fri 19:10 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>d10 Sat 01:30 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>d10 Sat 11:30 Jefferson Lines: Billings -&gt; Whitefish</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>d10 Sat 10:45 Northwestern Stage Lines</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>d14 Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>d10 Sat 11:10 FlixBus-us: Spokane Station -&gt; Pasco Bus Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>d10 Sat 13:25 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>d11 Sun 04:45 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>d11 Sun 10:30 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>d11 Sun 14:00 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>d11 Sun 18:43 Amtrak</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>wait 1 day(s): the same buses run, everything shifts 24 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>d13 Tue 03:00 BeeLine Express-Village Travel</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Oklahoma (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>d14 Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>d13 Tue 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>d13 Tue 08:25 Amtrak</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>d13 Tue 11:35 Greyhound-us: Oklahoma City Bus Station -&gt; Ft Worth Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>d13 Tue 14:23 Amtrak</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Longview</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>d13 Tue 16:35 Greyhound-us: Ft Worth Bus Station -&gt; Dallas Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>d13 Tue 18:30 Amtrak Chartered Vehicle</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Longview</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Shreveport Sportran Intermodal Terminal</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>d14 Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>d13 Tue 19:15 Greyhound-us: Longview Bus Station -&gt; Shreveport Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>d13 Tue 20:50 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Shreveport Bus Station</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>d15 Thu 20:25</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>d14 Wed 08:35 Greyhound-us: Shreveport Bus Station -&gt; Dallas Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>d13 Tue 22:40 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:20</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>d14 Wed 06:55 Greyhound-us: Texarkana (Travel Stop) -&gt; Memphis Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>d14 Wed 05:45 On foot (Big River Crossing, open 06:00-22:00)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:20</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>d14 Wed 05:55 On foot (Big River Crossing, open 06:00-22:00): Memphis -&gt; Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>d14 Wed 06:30 On foot (Big River Crossing, open 06:00-22:00)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:20</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>d14 Wed 06:40 On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing (on foot from Memphis Amtrak) -&gt; Memphis</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>d14 Wed 07:21 MATA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2ND STREET at VANCE AVENUE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>AIRWAYS TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:20</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>d14 Wed 07:52 MATA: ADAMS AVENUE at 4TH STREET -&gt; WILLIAM HUDSON TRANSIT CENTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>d14 Wed 09:00 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Birmingham Intermodal Facility</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>d15 Thu 16:20</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>d14 Wed 21:20 Greyhound-us: Memphis Bus Station -&gt; Atlanta Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>d14 Wed 13:50 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Birmingham Intermodal Facility</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>d15 Thu 10:50</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>d14 Wed 16:15 Greyhound-us: Birmingham Intermodal Facility -&gt; Atlanta Bus Station</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>leg</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>why it needs checking</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source / assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>d5 Mon 06:40 Hanover (Hanover Inn) -&gt; Boston South Station</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hand-entered (Dartmouth Coach): confirm times and days on the carrier site</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Hanover -&gt; Boston South Station 06:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>d7 Wed 18:57 Museum Campus/11th St. -&gt; Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>router local-transit proxy: plan the real bus, walk or taxi</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>South Shore into Chicago. To the Chicago bus station: walk or CTA (2 km), 4.7 h to spare before the 22:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>d10 Sat 10:45 Spokane -&gt; Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>hand-entered (Northwestern Stage Lines): confirm times and days on the carrier site</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NWL 710 Spokane -&gt; Pasco</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>d11 Sun 02:30 Salt Lake City Intermodal Trans Ctr -&gt; Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>router local-transit proxy: plan the real bus, walk or taxi</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Arrive SLC Intermodal 02:30; the Salt Lake Express leaves from the airport at 04:45. No transit at that hour: taxi, or walk 6.8 km (~90 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>d11 Sun 04:45 Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>hand-entered (Salt Lake Express): confirm times and days on the carrier site</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SLE 7021 Salt Lake City (Airport) 04:45 -&gt; Saint George (Bluff St Office) 10:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>d11 Sun 10:30 Saint George (Bluff St Office) -&gt; Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>hand-entered (Salt Lake Express): confirm times and days on the carrier site</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SLE 8035 Saint George (Bluff St Office) 10:30 -&gt; Las Vegas (Airport) 11:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>d11 Sun 11:40 Las Vegas (Airport) -&gt; Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>router local-transit proxy: plan the real bus, walk or taxi</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Airport to downtown terminal: RTC bus (4 km), 2.3 h to spare before the 14:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>d14 Wed 03:45 Memphis Bus Station -&gt; Memphis</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>router local-transit proxy: plan the real bus, walk or taxi</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Real weekday MATA (the router shows a local-transit proxy here): Walker 04:30 Airways Transit Center -&gt; Vance &amp; 3rd 05:21, walk 13 min to Central Station for the 05:45 bridge walk. Backup: route 12 Airways 05:14 -&gt; Florida &amp; Georgia 05:51, walk 19 min to the bridge. Saturday has no service this early.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>d14 Wed 05:45 Memphis -&gt; Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>hand-entered (On foot (Big River Crossing, open 06:00-22:00)): confirm times and days on the carrier site</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Memphis Amtrak -&gt; Arkansas line on Big River Crossing (walk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>d14 Wed 06:30 Arkansas line on Big River Crossing (on foot from Memphis Amtrak) -&gt; Memphis</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>hand-entered (On foot (Big River Crossing, open 06:00-22:00)): confirm times and days on the carrier site</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing -&gt; Memphis Amtrak (walk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>All GTFS legs</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>feeds are a snapshot (Sep-Oct 2026): re-check every once-daily leg on the carrier site before booking</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Greyhound, Flix, Jefferson, Barons, Amtrak</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Four Winds shuttle (alternative to the Michiana run)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>return arrival times in Chicago are not published (assumed 1 h 40 min); 21+ with photo ID</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>fourwindscasinoshuttle.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>date (Monday start)</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>depart</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>arrive</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>carrier</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>day 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mon 09:30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Dartmouth Coach</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Hanover -&gt; Boston South Station 06:40</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>dartmouthcoach.com (reserve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>day 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mon 11:55</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Portland, ME to/from Boston &amp; Logan Airport</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>day 1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mon 14:25</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Portland, ME to/from Boston &amp; Logan Airport</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>day 1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mon 22:22</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Amtrak</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Acela</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Amtrak (reserved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>day 2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tue Sep 29</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Tue 11:25</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FlixBus-us</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NYC Chinatown - Atlanta</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>day 2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tue Sep 29</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Tue 13:55</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Atlanta - Columbia - Raleigh (Subsidy)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>day 2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tue Sep 29</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Camden (McDonald's)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Tue 16:55</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Charlotte Bus Station</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Raleigh - Jacksonville</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>day 2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tue Sep 29</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Wed 04:30</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Barons Bus Lines</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Charlotte -&gt; Columbus</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>day 3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wed Sep 30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Wed 12:20</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Michigan City</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Barons Bus Lines</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Columbus (E Mound St) -&gt; Chicago</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>day 3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wed Sep 30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Thu 06:20</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Chicago - Milwaukee - Minneapolis</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>day 4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Thu Oct 01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Thu 14:55</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Minneapolis -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>day 4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Thu Oct 01</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Thu 19:50</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Fargo -&gt; Sioux Falls</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>day 4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Thu Oct 01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Fri 02:15</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Sioux Falls -&gt; Kansas City</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>day 5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Fri Oct 02</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>03:25</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Fri 10:05</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Kansas City -&gt; Sioux Falls</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>day 5</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Fri Oct 02</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sat 00:25</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Minneapolis -&gt; Billings</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>day 6</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sat Oct 03</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sat 10:30</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Billings -&gt; Spokane</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>day 6</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sat Oct 03</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sat 13:10</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Northwestern Stage Lines</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NWL 710 Spokane -&gt; Pasco</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>day 6</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sat Oct 03</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sun 02:30</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Seattle-Boise-SLC-Denver</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>day 7</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sun Oct 04</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sun 10:20</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>SLE 7021 Salt Lake City (Airport) 04:45 -&gt; Saint George (Bluff St Office) 10:20</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>saltlakeexpress.com (reserve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>day 7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sun Oct 04</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sun 11:40</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>SLE 8035 Saint George (Bluff St Office) 10:30 -&gt; Las Vegas (Airport) 11:40</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>saltlakeexpress.com (reserve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>day 7</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sun Oct 04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sun 18:15</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Los Angeles - Las Vegas</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>day 7</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sun Oct 04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tue 01:47</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Amtrak</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Southwest Chief</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Amtrak (reserved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>day 9</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tue Oct 06</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Tue 06:38</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Oklahoma (Amtrak)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>BeeLine Express-Village Travel</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak) -&gt; Oklahoma City</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>BeeLine (phone/site)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>day 9</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Tue Oct 06</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Tue 12:27</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Amtrak</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Heartland Flyer</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Amtrak (reserved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>day 9</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Tue Oct 06</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>14:23</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Tue 18:18</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Longview</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Amtrak</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Texas Eagle</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Amtrak (reserved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>day 9</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Tue Oct 06</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Longview</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Tue 19:50</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Shreveport Sportran Intermodal Terminal</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Amtrak Chartered Vehicle</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Amtrak Thruway Connecting Service</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Amtrak (reserved)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>day 9</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Tue Oct 06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Shreveport Bus Station</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Tue 22:10</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Texarkana - Houston</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>day 9</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tue Oct 06</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>22:40</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Texarkana (Travel Stop)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Wed 03:45</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Dallas - Nashville - Detroit</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>day 10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Wed Oct 07</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Memphis Bus Station</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Wed 13:25</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Birmingham Intermodal Facility</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Atlanta - Memphis</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>day 10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wed Oct 07</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Birmingham Intermodal Facility</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Wed 20:25</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Greyhound-us</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Nashville - Tallahassee</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>carrier site / app</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Walk-up / local (no reservation): Advance Transit, MATA, Michigan City Transit, South Shore Line (ticket at station or app), Houston METRO, JTA, RTC Las Vegas, UTA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HT Book ahead: dates for a Monday Oct 26 start, price and segment-booked columns with totals, DST note
Clocks fall back Sun Nov 1 (day 7); the Pasco -> Salt Lake overnight runs through it and elapsed comes
to ~231.1 h with schedules on local time.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ht_itinerary.xlsx
+++ b/docs/ht_itinerary.xlsx
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -77,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -91,6 +93,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4706,7 +4710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4718,6 +4722,8 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4728,7 +4734,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>date (Monday start)</t>
+          <t>date (start Mon Oct 26)</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -4764,6 +4770,16 @@
       <c r="I1" s="2" t="inlineStr">
         <is>
           <t>book</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>segment booked</t>
         </is>
       </c>
     </row>
@@ -4775,7 +4791,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mon Sep 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4813,6 +4829,7 @@
           <t>dartmouthcoach.com (reserve)</t>
         </is>
       </c>
+      <c r="J2" s="9" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4822,7 +4839,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mon Sep 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4860,6 +4877,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J3" s="9" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4869,7 +4887,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mon Sep 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4907,6 +4925,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4916,7 +4935,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mon Sep 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4954,6 +4973,7 @@
           <t>Amtrak (reserved)</t>
         </is>
       </c>
+      <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4963,7 +4983,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tue Sep 29</t>
+          <t>Tue Oct 27</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5001,6 +5021,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5010,7 +5031,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tue Sep 29</t>
+          <t>Tue Oct 27</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5048,6 +5069,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5057,7 +5079,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tue Sep 29</t>
+          <t>Tue Oct 27</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5095,6 +5117,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5104,7 +5127,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tue Sep 29</t>
+          <t>Tue Oct 27</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5142,6 +5165,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5151,7 +5175,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wed Sep 30</t>
+          <t>Wed Oct 28</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5189,6 +5213,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5198,7 +5223,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Wed Sep 30</t>
+          <t>Wed Oct 28</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5236,6 +5261,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5245,7 +5271,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Thu Oct 01</t>
+          <t>Thu Oct 29</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5283,6 +5309,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5292,7 +5319,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Thu Oct 01</t>
+          <t>Thu Oct 29</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -5330,6 +5357,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5339,7 +5367,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Thu Oct 01</t>
+          <t>Thu Oct 29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5377,6 +5405,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5386,7 +5415,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fri Oct 02</t>
+          <t>Fri Oct 30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5424,6 +5453,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5433,7 +5463,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fri Oct 02</t>
+          <t>Fri Oct 30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5471,6 +5501,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5480,7 +5511,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sat Oct 03</t>
+          <t>Sat Oct 31</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5518,6 +5549,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5527,7 +5559,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sat Oct 03</t>
+          <t>Sat Oct 31</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5565,6 +5597,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5574,7 +5607,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sat Oct 03</t>
+          <t>Sat Oct 31</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5612,6 +5645,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5621,7 +5655,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sun Oct 04</t>
+          <t>Sun Nov 01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5659,6 +5693,7 @@
           <t>saltlakeexpress.com (reserve)</t>
         </is>
       </c>
+      <c r="J20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5668,7 +5703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sun Oct 04</t>
+          <t>Sun Nov 01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5706,6 +5741,7 @@
           <t>saltlakeexpress.com (reserve)</t>
         </is>
       </c>
+      <c r="J21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5715,7 +5751,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sun Oct 04</t>
+          <t>Sun Nov 01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5753,6 +5789,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5762,7 +5799,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sun Oct 04</t>
+          <t>Sun Nov 01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5800,6 +5837,7 @@
           <t>Amtrak (reserved)</t>
         </is>
       </c>
+      <c r="J23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5809,7 +5847,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tue Oct 06</t>
+          <t>Tue Nov 03</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5847,6 +5885,7 @@
           <t>BeeLine (phone/site)</t>
         </is>
       </c>
+      <c r="J24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5856,7 +5895,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tue Oct 06</t>
+          <t>Tue Nov 03</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5894,6 +5933,7 @@
           <t>Amtrak (reserved)</t>
         </is>
       </c>
+      <c r="J25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5903,7 +5943,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tue Oct 06</t>
+          <t>Tue Nov 03</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5941,6 +5981,7 @@
           <t>Amtrak (reserved)</t>
         </is>
       </c>
+      <c r="J26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5950,7 +5991,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tue Oct 06</t>
+          <t>Tue Nov 03</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5988,6 +6029,7 @@
           <t>Amtrak (reserved)</t>
         </is>
       </c>
+      <c r="J27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5997,7 +6039,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tue Oct 06</t>
+          <t>Tue Nov 03</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -6035,6 +6077,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6044,7 +6087,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tue Oct 06</t>
+          <t>Tue Nov 03</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -6082,6 +6125,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6091,7 +6135,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Wed Oct 07</t>
+          <t>Wed Nov 04</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6129,6 +6173,7 @@
           <t>carrier site / app</t>
         </is>
       </c>
+      <c r="J30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6138,7 +6183,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Wed Oct 07</t>
+          <t>Wed Nov 04</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6176,12 +6221,52 @@
           <t>carrier site / app</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Walk-up / local (no reservation): Advance Transit, MATA, Michigan City Transit, South Shore Line (ticket at station or app), Houston METRO, JTA, RTC Las Vegas, UTA</t>
+      <c r="J31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="J32" s="10">
+        <f>SUM(J2:J31)</f>
+        <v/>
+      </c>
+      <c r="K32" s="2">
+        <f>COUNTA(K2:K31)&amp;" of 30 booked"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Walk-up / local (no reservation): MATA, Michigan City Transit, South Shore Line (ticket at station or app), Houston METRO, JTA, RTC Las Vegas, UTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DST: clocks fall back Sun Nov 1 02:00 (day 7 of a Mon Oct 26 start). The Pasco -&gt; Salt Lake overnight Greyhound runs through it (due 02:30 local); schedules keep local times, so elapsed is ~231.1 h, not 230.10. Confirm that night with the carriers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Dates are trips from the timetable window (Sep 28 start) relabelled to a Mon Oct 26 start: confirm each leg runs on its date when pricing.</t>
         </is>
       </c>
     </row>

</xml_diff>